<commit_message>
test: temporarily exercise non-default action.yml inputs live
Passes comment: false, job-summary: true, max-rows-per-sheet: 1,
diff-mode: coordinate to this PR's own xlsx-diff.yml call, and modifies
the already-merged smoke-test fixture (3 real cell changes) so this
run gets a genuine Modified status against master rather than Added.
Adds a temporary step printing has-changes/changed-files-count. To be
reverted once the run is confirmed.
</commit_message>
<xml_diff>
--- a/tests/fixtures/normal/_action_smoke_test_tmp.xlsx
+++ b/tests/fixtures/normal/_action_smoke_test_tmp.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,22 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,9 +417,19 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Grade</t>
         </is>
       </c>
     </row>
@@ -440,11 +440,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>S</t>
         </is>
       </c>
     </row>
@@ -457,11 +457,6 @@
       <c r="B3" t="n">
         <v>90</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -470,18 +465,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>